<commit_message>
Implemented workforce reporting pipeline with LLM insights
</commit_message>
<xml_diff>
--- a/data/Wohlig Active Employee Data.xlsx
+++ b/data/Wohlig Active Employee Data.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="128">
   <si>
     <t>WOHLIG PROJECT DASHBOARD</t>
   </si>
@@ -290,6 +290,18 @@
     <t>Projects</t>
   </si>
   <si>
+    <t>Aiman Ansari</t>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>Pocket Stdio</t>
+  </si>
+  <si>
+    <t>Wajid</t>
+  </si>
+  <si>
     <t>Sr No.</t>
   </si>
   <si>
@@ -396,25 +408,18 @@
     <t>Closed</t>
   </si>
   <si>
-    <t>ankit.shrivastav@wohlig.com</t>
+    <t>Weekly Automation Task</t>
   </si>
   <si>
-    <t>Aryan Gupta
-Dhruv Solanki
-Krishank Daga
-Nishita Patel
-Parth Gala</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Weekly Automation Task</t>
+    <t>ankit.shrivastav@wohlig.com</t>
   </si>
   <si>
     <t xml:space="preserve">Shubham Jain
 Shubham Satpute
 </t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
   <si>
     <t>E-mail Automation</t>
@@ -635,7 +640,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -733,6 +738,12 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="2" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="3" fillId="8" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
@@ -13896,18 +13907,38 @@
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
+      <c r="A2" s="35">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="36">
+        <v>46163.0</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="14"/>
+      <c r="A3" s="24">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="36">
+        <v>46163.0</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="17"/>
@@ -14991,90 +15022,90 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B1" s="36" t="s">
-        <v>88</v>
-      </c>
-      <c r="C1" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="E1" s="36" t="s">
+      <c r="A1" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="B1" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="C1" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="D1" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="I1" s="36" t="s">
+      <c r="E1" s="38" t="s">
         <v>95</v>
       </c>
+      <c r="F1" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="G1" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="I1" s="38" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="37">
+      <c r="A2" s="39">
         <v>1.0</v>
       </c>
-      <c r="B2" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="38" t="s">
+      <c r="B2" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="38" t="s">
-        <v>97</v>
-      </c>
-      <c r="F2" s="39" t="s">
-        <v>98</v>
-      </c>
-      <c r="G2" s="40">
+      <c r="E2" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="G2" s="42">
         <v>46132.0</v>
       </c>
-      <c r="H2" s="40">
+      <c r="H2" s="42">
         <v>46173.0</v>
       </c>
-      <c r="I2" s="41" t="s">
-        <v>99</v>
+      <c r="I2" s="43" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="38">
+      <c r="A3" s="40">
         <v>2.0</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="D3" s="41" t="s">
+      <c r="C3" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="41" t="s">
-        <v>101</v>
-      </c>
-      <c r="F3" s="41" t="s">
-        <v>102</v>
-      </c>
-      <c r="G3" s="40">
+      <c r="E3" s="43" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="42">
         <v>46168.0</v>
       </c>
-      <c r="H3" s="40">
+      <c r="H3" s="42">
         <v>46290.0</v>
       </c>
-      <c r="I3" s="41" t="s">
-        <v>103</v>
+      <c r="I3" s="43" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -16082,137 +16113,137 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="42" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="D1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="G1" s="42" t="s">
-        <v>106</v>
-      </c>
-      <c r="H1" s="42" t="s">
-        <v>95</v>
+      <c r="B1" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="44" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" s="44" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="44" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" s="44" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" s="44" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="45" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="46">
+        <v>46062.0</v>
+      </c>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="41" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="45" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="45" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="46">
+        <v>46168.0</v>
+      </c>
+      <c r="F3" s="46"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="43" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="43" t="s">
-        <v>108</v>
-      </c>
-      <c r="E2" s="44">
-        <v>46062.0</v>
-      </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="43" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" s="41" t="s">
-        <v>109</v>
-      </c>
-      <c r="C3" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="43" t="s">
-        <v>110</v>
-      </c>
-      <c r="E3" s="44">
-        <v>46168.0</v>
-      </c>
-      <c r="F3" s="44"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>111</v>
-      </c>
-      <c r="C4" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="43" t="s">
-        <v>112</v>
-      </c>
-      <c r="E5" s="47">
+      <c r="D5" s="45" t="s">
+        <v>116</v>
+      </c>
+      <c r="E5" s="49">
         <v>46071.0</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46" t="s">
-        <v>103</v>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="48" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="s">
+      <c r="A6" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="46" t="s">
-        <v>113</v>
-      </c>
-      <c r="D6" s="46" t="s">
+      <c r="C6" s="48" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="48" t="s">
         <v>35</v>
       </c>
       <c r="E6" s="13">
         <v>46062.0</v>
       </c>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="46" t="s">
-        <v>103</v>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="48" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -17219,134 +17250,113 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="48" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="48" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="48" t="s">
-        <v>90</v>
-      </c>
-      <c r="D1" s="48" t="s">
-        <v>91</v>
-      </c>
-      <c r="E1" s="48" t="s">
+      <c r="A1" s="50" t="s">
         <v>92</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="B1" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="48" t="s">
+      <c r="C1" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="H1" s="48" t="s">
+      <c r="D1" s="50" t="s">
         <v>95</v>
       </c>
+      <c r="E1" s="50" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1" s="50" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="H1" s="50" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="38" t="s">
-        <v>114</v>
-      </c>
-      <c r="C2" s="38" t="s">
+      <c r="B2" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="E2" s="38" t="s">
-        <v>116</v>
-      </c>
-      <c r="F2" s="44">
+      <c r="D2" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="F2" s="46">
         <v>45852.0</v>
       </c>
-      <c r="G2" s="44">
+      <c r="G2" s="46">
         <v>46162.0</v>
       </c>
-      <c r="H2" s="38" t="s">
-        <v>117</v>
+      <c r="H2" s="40" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="49" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="49" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" s="49" t="s">
+      <c r="A3" s="51" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3" s="51" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="51" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="D3" s="51" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="F3" s="52">
+        <v>46174.0</v>
+      </c>
+      <c r="G3" s="53">
+        <v>46189.0</v>
+      </c>
+      <c r="H3" s="51" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="51" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="E3" s="49" t="s">
+      <c r="C4" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="51" t="s">
         <v>119</v>
       </c>
-      <c r="F3" s="50">
+      <c r="E4" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="F4" s="52">
         <v>46174.0</v>
       </c>
-      <c r="G3" s="51">
+      <c r="G4" s="53">
         <v>46189.0</v>
       </c>
-      <c r="H3" s="49" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="49" t="s">
-        <v>121</v>
-      </c>
-      <c r="B4" s="49" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="49" t="s">
-        <v>118</v>
-      </c>
-      <c r="E4" s="49" t="s">
-        <v>122</v>
-      </c>
-      <c r="F4" s="50">
-        <v>46174.0</v>
-      </c>
-      <c r="G4" s="51">
-        <v>46189.0</v>
-      </c>
-      <c r="H4" s="49" t="s">
-        <v>120</v>
+      <c r="H4" s="51" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="49" t="s">
-        <v>114</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="49" t="s">
-        <v>115</v>
-      </c>
-      <c r="E5" s="52" t="s">
-        <v>124</v>
-      </c>
-      <c r="F5" s="50">
-        <v>46174.0</v>
-      </c>
-      <c r="G5" s="51">
-        <v>46189.0</v>
-      </c>
-      <c r="H5" s="49" t="s">
-        <v>120</v>
-      </c>
+      <c r="E5" s="54"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="53"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>

</xml_diff>